<commit_message>
Publish five evergreen journaling tutorials
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J142"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6929,6 +6929,266 @@
       <c r="J142" t="inlineStr">
         <is>
           <t>how-to-make-a-junk-journal-from-an-old-book</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>How to Glue Thin Paper Without Wrinkles</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>lead magnet tutorial</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Evergreen beginner technique</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0004_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Five adhesive methods by paper type</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>how-to-glue-thin-paper-without-wrinkles</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>One Envelope, Five Junk Journal Pockets</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>lead magnet tutorial</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Evergreen paper engineering</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0013_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Five functional envelope transformations</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>one-envelope-five-junk-journal-pockets</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>The Three-Layer Ephemera Cluster Formula</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>lead magnet tutorial</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Evergreen composition</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0010_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Base-story-accent formula</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>three-layer-ephemera-cluster-formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>12 Tiny Journal Challenges for Days You Feel Stuck</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>listing-allocated slot resolved to lead tutorial</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Evergreen creative block</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0022_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>No eligible verified unused listing; product bridge intentionally omitted</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>12-tiny-journal-challenges</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>How to Turn One Photo into a Memory Page</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>listing-allocated slot resolved to lead tutorial</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Evergreen memory keeping</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0017_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>No eligible verified unused listing; product bridge intentionally omitted</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>one-photo-to-one-memory-page</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish five mistakes and palette articles
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J147"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7189,6 +7189,266 @@
       <c r="J147" t="inlineStr">
         <is>
           <t>one-photo-to-one-memory-page</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>8 Junk Journal Pocket Mistakes to Avoid</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>lead magnet tutorial</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Evergreen pockets and tucks</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0013_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Audience: journal makers; hook: pockets that catch or fail; target query: junk journal pocket mistakes</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>8-junk-journal-pocket-mistakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>7 Card Layering Mistakes That Make Cards Look Crooked</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>lead magnet tutorial</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Evergreen card construction</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0006_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Audience: card makers; hook: cleaner mats and layers; target query: card layering mistakes</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>7-card-layering-mistakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>9 Scrapbooking Mistakes That Hide the Story</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>lead magnet tutorial</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Evergreen scrapbook composition</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0017_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Audience: memory keepers; hook: put the story back first; target query: scrapbooking mistakes</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>9-scrapbooking-mistakes-that-hide-the-story</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>8 Printable Paper Craft Mistakes That Waste Ink and Paper</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>listing-allocated slot resolved to lead tutorial</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Evergreen printable craft technique</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0010_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>No eligible source-verified unused listing; audience: printable crafters; target query: printable paper mistakes</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>8-printable-paper-mistakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>5 Dusty Blue Palettes for Vintage Paper Crafts</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>listing-allocated slot resolved to lead palette</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Evergreen vintage color palette</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0004_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>No eligible source-verified unused listing; five general-use palette recipes with hex values</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>5-dusty-blue-palettes-for-vintage-paper-crafts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish five Thanksgiving keepsake articles
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J152"/>
+  <dimension ref="A1:J157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7449,6 +7449,266 @@
       <c r="J152" t="inlineStr">
         <is>
           <t>5-dusty-blue-palettes-for-vintage-paper-crafts</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>A Thankful-for-You Card with 12 Specific Things to Say</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Thanksgiving gratitude card</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>4568614719</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0006_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Target query: thanksgiving thank you card ideas; optional Autumn Dreams listing, unused and live</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>thank-you-card-12-specific-things</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>A Thanksgiving Gratitude Journal Page That Feels Honest</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Thanksgiving gratitude journaling</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>4565499542</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0022_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Target query: thanksgiving gratitude journal page; optional Autumn Harvest listing, unused and live</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>honest-thanksgiving-gratitude-journal-page</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>A One-Photo Thanksgiving Table Scrapbook Page</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Thanksgiving scrapbooking</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>4550255539</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0017_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Target query: thanksgiving scrapbook page ideas; optional Country Kitchen listing, unused and live</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>one-photo-thanksgiving-table-scrapbook-page</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Thanksgiving Place Cards Guests Can Keep</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>listing-bound useful project</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Thanksgiving card making</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>4570200856</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0022_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Target query: thanksgiving place card keepsake; optional Autumn Leaves listing, unused and live</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>thanksgiving-place-cards-guests-can-keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>A Thanksgiving Family Memory Folio in Six Folds</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>listing-bound useful project</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Thanksgiving memory keeping</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>4550255395</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>perfect-workplace_0010_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>approved-codex + branding</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Target query: thanksgiving memory folio; optional Old Barn listing, unused and live</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>thanksgiving-family-memory-folio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 20 fall and winter memory-keeping articles
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J157"/>
+  <dimension ref="A1:J177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7709,6 +7709,746 @@
       <c r="J157" t="inlineStr">
         <is>
           <t>thanksgiving-family-memory-folio</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>A Cozy Reading-Night Pocket Page</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>tutorial</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>a-cozy-reading-night-pocket-page</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>7 Fall Scrapbook Mistakes That Make Pages Feel Busy</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>mistakes infographic</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>fall-scrapbook-mistakes-that-make-pages-feel-busy</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>12 Things to Save From Thanksgiving Weekend</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>iPhone Notes</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>things-to-save-from-thanksgiving-weekend</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Cranberry, Sage, Pecan and Linen for Thanksgiving Pages</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>palette</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>cranberry-sage-pecan-and-linen-for-thanksgiving-pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>A Calm Snow-Day Memory Page in Five Steps</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>tutorial</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>a-calm-snow-day-memory-page</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>8 Christmas Scrapbook Mistakes That Hide the Story</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>mistakes infographic</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>christmas-scrapbook-mistakes-that-hide-the-story</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>15 Tiny Christmas-Eve Details to Write Down</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>iPhone Notes</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>tiny-christmas-eve-details-to-write-down</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Pine, Cranberry, Candle Gold and Cream for Christmas Pages</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>palette</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>pine-cranberry-candle-gold-and-cream-christmas-palette</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>A No-Stress Holiday Photo Pocket</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>tutorial</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>a-no-stress-holiday-photo-pocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>7 Winter Journal Mistakes That Make Pages Feel Cold</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>mistakes infographic</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>winter-journal-mistakes-that-make-pages-feel-cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>14 Things to Journal Between Christmas and New Year</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>iPhone Notes</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>things-to-journal-between-christmas-and-new-year</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Frost Blue, Wool, Pine and Berry for Winter Cabin Pages</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>palette</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>frost-blue-wool-pine-and-berry-winter-cabin-palette</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>A Gentle New-Year Reflection Spread</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>tutorial</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>a-gentle-new-year-reflection-spread</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>6 New-Year Journal Mistakes That Add Pressure</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>mistakes infographic</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>new-year-journal-mistakes-that-add-pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>12 Gentle January Journal Prompts for Winter Days</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>iPhone Notes</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>gentle-january-journal-prompts-for-winter-days</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Midnight, Parchment, Moon Gray and Gold for New-Year Pages</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>palette</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>midnight-parchment-moon-gray-and-gold-new-year-palette</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>A 10-Minute Winter Collage for Stressful Days</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>tutorial</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>a-ten-minute-winter-collage-for-stressful-days</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>7 Valentine Scrapbook Mistakes That Flatten Real Stories</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>mistakes infographic</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>valentine-scrapbook-mistakes-that-flatten-real-stories</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>14 Valentine Memories Beyond Romance</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>iPhone Notes</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>valentine-memories-beyond-romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Dusty Rose, Oxblood, Cocoa and Ivory for Valentine Pages</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>palette</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>fall-winter seasonal memory keeping</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Requested 20-article alternating seasonal collection</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>dusty-rose-oxblood-cocoa-and-ivory-valentine-palette</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish five evergreen conversion articles
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J177"/>
+  <dimension ref="A1:J182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8449,6 +8449,222 @@
       <c r="J177" t="inlineStr">
         <is>
           <t>dusty-rose-oxblood-cocoa-and-ivory-valentine-palette</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>A One-Day Fold-Out Timeline for Your Journal</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>tutorial</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>evergreen memory keeping</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>approved-codex/make-a-page-feel-like-a-place.jpg</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Lead article; conversion CTA + 3 designed pins</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>a-one-day-fold-out-timeline-for-your-journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Scrapbook Caption Mistakes That Make Memories Sound Generic</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>avoiding mistakes infographic</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>evergreen memory keeping</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>approved-codex/make-a-page-feel-like-a-place.jpg</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Lead article; conversion CTA + 3 designed pins</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>scrapbook-caption-mistakes-that-make-memories-sound-generic</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Things to Write Down After a Good Conversation</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>iPhone Notes</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>evergreen reflective journaling</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Lead article; authentic iPhone Notes + 3 designed pins</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>things-to-write-down-after-a-good-conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Ink, Oat, Clay and Moss for Grounded Journal Pages</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>palette</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>evergreen color palette</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>ledger-textile-junk-journal-palette-ideas</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Lead article; real listing page palette + 3 designed pins</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>ink-oat-clay-and-moss-for-grounded-journal-pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Turn a Voice Note Into a Memory Page</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>tutorial</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>evergreen memory keeping</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>approved-codex/make-a-page-feel-like-a-place.jpg</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Lead article; conversion CTA + 3 designed pins</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>turn-a-voice-note-into-a-memory-page</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add relevant product bridges to five articles
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -8473,8 +8473,11 @@
           <t>evergreen memory keeping</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr"/>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>110_Old_Pages</t>
+        </is>
+      </c>
       <c r="G178" t="inlineStr">
         <is>
           <t>approved-codex/make-a-page-feel-like-a-place.jpg</t>
@@ -8482,7 +8485,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Lead article; conversion CTA + 3 designed pins</t>
+          <t>Lead article; conversion CTA + 3 designed pins; Live topic-matched listing embedded in article.</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -8517,8 +8520,11 @@
           <t>evergreen memory keeping</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr"/>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>212_Ledger_Pages</t>
+        </is>
+      </c>
       <c r="G179" t="inlineStr">
         <is>
           <t>approved-codex/make-a-page-feel-like-a-place.jpg</t>
@@ -8526,7 +8532,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Lead article; conversion CTA + 3 designed pins</t>
+          <t>Lead article; conversion CTA + 3 designed pins; Live topic-matched listing embedded in article.</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -8561,12 +8567,14 @@
           <t>evergreen reflective journaling</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>117_Morning_Brew</t>
+        </is>
+      </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Lead article; authentic iPhone Notes + 3 designed pins</t>
+          <t>Lead article; authentic iPhone Notes + 3 designed pins; Live topic-matched listing embedded in article.</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -8603,14 +8611,12 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>ledger-textile-junk-journal-palette-ideas</t>
-        </is>
-      </c>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr"/>
+          <t>202_Ledger_Textile</t>
+        </is>
+      </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Lead article; real listing page palette + 3 designed pins</t>
+          <t>Lead article; real listing page palette + 3 designed pins; Live topic-matched listing embedded in article.</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -8645,8 +8651,11 @@
           <t>evergreen memory keeping</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
-      <c r="F182" t="inlineStr"/>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>186_Old_Song</t>
+        </is>
+      </c>
       <c r="G182" t="inlineStr">
         <is>
           <t>approved-codex/make-a-page-feel-like-a-place.jpg</t>
@@ -8654,7 +8663,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Lead article; conversion CTA + 3 designed pins</t>
+          <t>Lead article; conversion CTA + 3 designed pins; Live topic-matched listing embedded in article.</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">

</xml_diff>

<commit_message>
Publish ten evergreen journal articles
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J182"/>
+  <dimension ref="A1:J192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8674,6 +8674,476 @@
       <c r="J182" t="inlineStr">
         <is>
           <t>turn-a-voice-note-into-a-memory-page</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>How to Keep One Ordinary Weekday Without Documenting Everything</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Memory Keeping</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>4577423256</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>how-to-keep-one-ordinary-weekday-without-documenting-everything</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>How to Write About a Hard Day Without Turning It Into an Essay</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Gentle Journaling</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>4506313481</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>how-to-write-about-a-hard-day-without-turning-it-into-an-essay</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>A Five-Minute Bedside Journal Ritual for Tired Nights</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Creative Rituals</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>4568645714</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>a-five-minute-bedside-journal-ritual-for-tired-nights</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>How to Make a Walk Memory Page From One Small Trace</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Memory Keeping</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>4525676610</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>how-to-make-a-walk-memory-page-from-one-small-trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>How to Journal a Memory You Can Hear but Cannot Picture</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Memory Keeping</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>4516818567</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>how-to-journal-a-memory-you-can-hear-but-cannot-picture</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>How to Return to an Unfinished Journal Page Without Starting Over</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>lead magnet with end listing</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Junk Journal Tutorials</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>4488065121</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>how-to-return-to-an-unfinished-journal-page-without-starting-over</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Antique Ledger Pages for a Family History Journal</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>listing-bound useful inspiration</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Junk Journal Inspiration</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>4568633117</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>antique-ledger-pages-for-a-family-history-journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>A Vintage Travel Journal That Begins Before the Trip</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>listing-bound useful inspiration</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Travel Journaling</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>4568281740</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>a-vintage-travel-journal-that-begins-before-the-trip</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>A Quiet Log Cabin Journal Theme for Nature Notes</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>listing-bound useful inspiration</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Junk Journal Inspiration</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>4567220885</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>a-quiet-log-cabin-journal-theme-for-nature-notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>A Colorful Dog Memory Journal That Still Feels Grown-Up</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>listing-bound useful inspiration</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Memory Keeping</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>4570186359</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>approved scene reference used in generated gen1</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>2026-10-03 evergreen batch; demand-first angle; live unused listing verified; critic PASS</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>a-colorful-dog-memory-journal-that-still-feels-grown-up</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ten journal articles with reviewed visuals
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J192"/>
+  <dimension ref="A1:J202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9144,6 +9144,426 @@
       <c r="J192" t="inlineStr">
         <is>
           <t>a-colorful-dog-memory-journal-that-still-feels-grown-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Keep the Story Behind Your Halloween Costume on Paper</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>lead-magnet · seasonal / educational</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Halloween memory keeping</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Spooky Gothic / 4568631116</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Audience: adults and families keeping costume memories; Hook: Remember why you chose it, not just how it looked; Target query: Halloween costume scrapbook ideas; tie=end; listing Spooky Gothic / 4568631116 freshly LIVE and UNUSED; Method: Three physical zones: The idea (why this costume), The making (sketch and tiny material trace), The night (one reaction or quote with date). Use one object-led process infographic.; Marketing ideation PASS (hook/intent/desire/path/save/voice/adfree/season &gt;=3). Seasonal=Halloween. Product language: commercial-use watercolor image collection, not clipart or templates. Final order AI disclosure &gt; paid bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>keep-the-story-behind-your-halloween-costume-on-paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Keep Your Wedding Dress Shopping Day in One Spread</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>lead-magnet · seasonal / educational</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Wedding-planning season</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Wedding Vintage / 4523625257</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Audience: sentimental brides after their dress appointment; Hook: Keep the feeling alongside the dress; Target query: wedding dress shopping scrapbook; tie=end; listing Wedding Vintage / 4523625257 freshly LIVE and UNUSED; Method: Three zones: Before the fitting (hope), The moment (photo or silhouette and words), What stayed (companions reaction and small detail). One object-led spread map.; Marketing ideation PASS (hook/intent/desire/path/save/voice/adfree/season &gt;=3). Seasonal=Wedding planning. Product language: commercial-use watercolor image collection, not clipart or templates. Final order AI disclosure &gt; paid bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>keep-your-wedding-dress-shopping-day-in-one-spread</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Make a Small Journal Desk That Packs Away in Minutes</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>lead-magnet · eternal / educational</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Dream workspace / cozy corner</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Neutral Tones / 4568645944</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Audience: small-space crafters using a shared table; Hook: Leave room for making and ordinary life; Target query: small space journaling setup; tie=end; listing Neutral Tones / 4568645944 freshly LIVE and UNUSED; Method: A portable working tray has an active sheet zone, tool cup, offcut envelope and flat drying place. Explain setup and shutdown, no invented claims that printables organize tools.; Marketing ideation PASS (hook/intent/desire/path/save/voice/adfree/season &gt;=3). Seasonal=eternal. Product language: commercial-use watercolor image collection, not clipart or templates. Final order AI disclosure &gt; paid bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>make-a-small-journal-desk-that-packs-away-in-minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Make a Garden Vision Page for the Life You Want</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>lead-magnet · eternal / educational</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Manifestation / dream-life journaling</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Dew Wisp / 4503796413</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Audience: aspiring slow-living gardeners; Hook: Picture a daily life you can actually begin; Target query: garden vision board journal; tie=end; listing Dew Wisp / 4503796413 freshly LIVE and UNUSED; Method: Three panels: Place (realistic desired corner), Daily feeling (one sensory detail), One action this week. Evergreen imagined garden, do not claim a current spring window or manifestation guarantees.; Marketing ideation PASS (hook/intent/desire/path/save/voice/adfree/season &gt;=3). Seasonal=eternal. Product language: commercial-use watercolor image collection, not clipart or templates. Final order AI disclosure &gt; paid bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>make-a-garden-vision-page-for-the-life-you-want</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Write a Letter to a Friend That Feels Like Being There</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>lead-magnet · eternal / educational</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Handmade cards / snail mail</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Love Letter / 4525663517</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Audience: friends keeping in touch over distance; Hook: Send a small piece of your everyday world; Target query: meaningful letter to a friend; tie=end; listing Love Letter / 4525663517 freshly LIVE and UNUSED; Method: Letter structure: one specific scene, one shared memory, one answerable question. Show a handwritten letter and small decorative enclosure, not mailing-service recommendations.; Marketing ideation PASS (hook/intent/desire/path/save/voice/adfree/season &gt;=3). Seasonal=eternal. Product language: commercial-use watercolor image collection, not clipart or templates. Final order AI disclosure &gt; paid bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>write-a-letter-to-a-friend-that-feels-like-being-there</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>A Plant-Care Journal That Remembers More Than Watering</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>lead-magnet · eternal / educational</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Bullet journal aesthetics</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Bloom Diary / 4511996030</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Audience: indoor plant keepers who enjoy a paper record; Hook: Notice how your little indoor garden changes; Target query: plant care journal ideas; tie=end; listing Bloom Diary / 4511996030 freshly LIVE and UNUSED; Method: One repeatable observation card: date, light position, visible leaf change, care already given, next observation. Avoid horticultural prescriptions or automatic watering schedules.; Marketing ideation PASS (hook/intent/desire/path/save/voice/adfree/season &gt;=3). Seasonal=eternal. Product language: commercial-use watercolor image collection, not clipart or templates. Final order AI disclosure &gt; paid bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>a-plant-care-journal-that-remembers-more-than-watering</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Gothic Journal Colors That Leave Room for Handwriting</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>listing-bound · eternal / spotlight</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Dark academia / vintage scholar</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Dark Manor / 4568148223</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Dark Manor 4568148223 freshly LIVE and UNUSED. Evergreen gothic architecture; educational listing spotlight. Three authentic non-character source pages, four role palettes, calm writing-space recipe. Product center; AI disclosure &gt; paid bridge &gt; optional freebie. Replaced patchwork Grunge Playing after visual gate. Marketing ideation PASS. No CSV.</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>gothic-journal-colors-that-leave-room-for-handwriting</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Folk Floral Journal Pages with a Handmade Rhythm</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>listing-bound · eternal / spotlight</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Cottagecore / slow living escape</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Folk Bloom / 4585952495</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Audience: crafters drawn to folk-art flowers and cottage-garden colors; Hook: Give your page the rhythm of something handmade; Target query: folk floral junk journal palette; tie=center; Folk Bloom / 4585952495 freshly LIVE and UNUSED; Method: Three authentic page palettes; repeat one floral shape at different scales, leave paper-colored space, anchor the composition with a single handwritten label. Preserve the folk-art feeling without covering every margin.; Marketing ideation PASS. Evergreen. Commercial-use watercolor IMAGE collection. Final AI disclosure &gt; product bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>folk-floral-journal-pages-with-a-handmade-rhythm</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Fairy Garden Journal Colors for an Airy Written Story</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>listing-bound · eternal / spotlight</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Romanticize your life / soft life</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Fairy Wings / 4585954090</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Audience: fairycore journalers seeking quiet woodland whimsy; Hook: Leave a little room for wonder; Target query: fairy garden junk journal palette; tie=center; Fairy Wings / 4585954090 freshly LIVE and UNUSED; Method: Three authentic non-character source page palettes; use pale paper as breathing space, one grounded woodland anchor, a gentle midtone and a real hero accent. Build a discovery page with a small observed-or-invented detail rather than an overfilled fantasy collage.; Marketing ideation PASS. Evergreen. Commercial-use watercolor IMAGE collection. Final AI disclosure &gt; product bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>fairy-garden-journal-colors-for-an-airy-written-story</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Build a Wizard Journal Around an Invented Place</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>listing-bound · eternal / spotlight</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Witchy / magic / grimoire</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Spell Cast / 4568281922</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Audience: fantasy writers making a paper world notebook; Hook: Make a place you can return to on paper; Target query: wizard fantasy journal ideas; tie=center; listing Spell Cast / 4568281922 freshly LIVE and UNUSED; Method: Three actual showpiece-page palettes; give invented place one landmark, one everyday rule and one resident note. Treat as creative writing, evergreen not Halloween or supernatural claims.; Marketing ideation PASS (hook/intent/desire/path/save/voice/adfree/season &gt;=3). Seasonal=eternal. Product language: commercial-use watercolor image collection, not clipart or templates. Final order AI disclosure &gt; paid bridge &gt; optional freebie. No CSV.</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>build-a-wizard-journal-around-an-invented-place</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ten winter and Christmas craft articles
</commit_message>
<xml_diff>
--- a/content_plan.xlsx
+++ b/content_plan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J202"/>
+  <dimension ref="A1:J212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9564,6 +9564,506 @@
       <c r="J202" t="inlineStr">
         <is>
           <t>build-a-wizard-journal-around-an-invented-place</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Make a Christmas Card With a Memory and a Wish</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>educational</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>4593150648</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>refs/infographics/approved-codex/make-a-page-feel-like-a-place.jpg; refs/branding/image.png</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=end; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>a-christmas-card-that-feels-personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>A Winter Window Journal Page for Early Dark Evenings</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>educational</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>4598839600</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>refs/infographics/approved-codex/make-a-page-feel-like-a-place.jpg; refs/branding/image.png</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=end; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>a-winter-window-journal-page-for-early-dark-evenings</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Build a Winter Letter Set With One Printable Collection</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>listing spotlight</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>4598839600</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=center; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>build-a-winter-letter-set-with-one-printable-collection</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Burgundy Plaid Christmas Cards Without Pattern Overload</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>listing spotlight</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>4593150648</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=center; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>burgundy-plaid-christmas-cards-without-pattern-overload</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Keep a Handwritten Christmas Recipe Without Hiding the Original</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>educational</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>4593150648</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>refs/infographics/approved-codex/make-a-page-feel-like-a-place.jpg; refs/branding/image.png</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=end; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>keep-a-handwritten-christmas-recipe-without-hiding-the-original</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Make Christmas Gift Tags That Match Handmade Cards</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>educational</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>4593150648</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>refs/infographics/approved-codex/make-a-page-feel-like-a-place.jpg; refs/branding/image.png</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=end; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>make-christmas-gift-tags-that-match-your-cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>A Snowflake Christmas Card That Becomes a Bookmark</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>listing spotlight</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>4593150728</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=center; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>snowflake-christmas-card-that-becomes-a-bookmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Make Tiny Advent Notes for Someone You Love This Christmas</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>educational</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>4593150648</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>refs/infographics/approved-codex/make-a-page-feel-like-a-place.jpg; refs/branding/image.png</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=end; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>tiny-advent-notes-for-someone-you-love</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Make Winter Happy Mail for Friends Who Live Far Away</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>educational</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>4598839600</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>refs/infographics/approved-codex/make-a-page-feel-like-a-place.jpg; refs/branding/image.png</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=end; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>winter-happy-mail-for-friends-far-away</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Make a Winter Reading Journal Cover With Breathing Room</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>listing spotlight</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Winter / Christmas / Holidays (explicit user request)</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>4593089360</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>refs/scenes/perfect-workplace_0013_originals.jpg; refs/scenes/perfect-workplace_0002_originals.jpg</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>2026-10-21 user explicitly requests all10 seasonal, overriding generic automatic calendar. Marketing ideation PASS; useful concrete paper project; tie=center; four seasonal IDs freshly LIVE verified via active Etsy catalog185 items and downloadable filenames. All four unused before batch; relevant intentional reuse within batch. Commercial-use watercolor image packs, no premade card/tag templates. Approved reference files included in generated graphics; no close winter mood scene reference existed, use saved cottage/window atmosphere anchors. Sources immutable. Full provenance and critique staging/article-batch-2026-10-21. No CSV requested.</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>winter-reading-journal-cover-with-breathing-room</t>
         </is>
       </c>
     </row>

</xml_diff>